<commit_message>
Update word list: 985 -> 1000 words
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dutch-words.xlsx
+++ b/dutch-words.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1972" uniqueCount="1937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1993">
   <si>
     <t>Dutch</t>
   </si>
@@ -5831,6 +5831,174 @@
   </si>
   <si>
     <t>1. the (bed)sheet; 2. tablecloth</t>
+  </si>
+  <si>
+    <t>1. indeed, really (modal particle, e.g. "ik denk het wel" = I do think so); 2. as many as (before a number, e.g. "wel duizend")</t>
+  </si>
+  <si>
+    <t>1. it; 2. the (before neuter/het-nouns)</t>
+  </si>
+  <si>
+    <t>1. over, about; 2. [om kwart ~ zeven] at quarter past seven; 3. left, remaining</t>
+  </si>
+  <si>
+    <t>really; real</t>
+  </si>
+  <si>
+    <t>perhaps, maybe</t>
+  </si>
+  <si>
+    <t>1. very (adverb); 2. whole, entire (adjective)</t>
+  </si>
+  <si>
+    <t>the hate, hatred</t>
+  </si>
+  <si>
+    <t>to grab, take, catch, catch hold of</t>
+  </si>
+  <si>
+    <t>1. seven; 2. [om kwart voor ~] at quarter to seven</t>
+  </si>
+  <si>
+    <t>to hit, to touch, to make contact with</t>
+  </si>
+  <si>
+    <t>(you) tell, narrate; (he) tells, narrates</t>
+  </si>
+  <si>
+    <t>the rest, relaxation, peace and quiet</t>
+  </si>
+  <si>
+    <t>de zomer</t>
+  </si>
+  <si>
+    <t>the summer</t>
+  </si>
+  <si>
+    <t>de winter</t>
+  </si>
+  <si>
+    <t>the winter</t>
+  </si>
+  <si>
+    <t>de lente</t>
+  </si>
+  <si>
+    <t>the spring (season)</t>
+  </si>
+  <si>
+    <t>de herfst</t>
+  </si>
+  <si>
+    <t>the autumn, fall</t>
+  </si>
+  <si>
+    <t>het weer</t>
+  </si>
+  <si>
+    <t>the weather</t>
+  </si>
+  <si>
+    <t>de winkel</t>
+  </si>
+  <si>
+    <t>the shop, store</t>
+  </si>
+  <si>
+    <t>de keuken</t>
+  </si>
+  <si>
+    <t>the kitchen</t>
+  </si>
+  <si>
+    <t>negen</t>
+  </si>
+  <si>
+    <t>nine</t>
+  </si>
+  <si>
+    <t>elf</t>
+  </si>
+  <si>
+    <t>eleven</t>
+  </si>
+  <si>
+    <t>twaalf</t>
+  </si>
+  <si>
+    <t>twelve</t>
+  </si>
+  <si>
+    <t>maandag</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>dinsdag</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>woensdag</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>donderdag</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>vrijdag</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>zaterdag</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>zondag</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>rood</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>blauw</t>
+  </si>
+  <si>
+    <t>blue</t>
+  </si>
+  <si>
+    <t>groen</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>geel</t>
+  </si>
+  <si>
+    <t>yellow</t>
+  </si>
+  <si>
+    <t>wit</t>
+  </si>
+  <si>
+    <t>white</t>
   </si>
 </sst>
 </file>
@@ -6174,7 +6342,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B986"/>
+  <dimension ref="A1:B1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="62.5" customWidth="1"/>
@@ -6306,7 +6474,7 @@
         <v>66</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>700</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -6370,7 +6538,7 @@
         <v>38</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>39</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -6439,10 +6607,10 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>38</v>
+        <v>1949</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>720</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -6722,7 +6890,7 @@
         <v>210</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>743</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
@@ -6898,7 +7066,7 @@
         <v>456</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>762</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
@@ -7370,7 +7538,7 @@
         <v>67</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>822</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
@@ -7498,7 +7666,7 @@
         <v>440</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>443</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.2">
@@ -7815,10 +7983,10 @@
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A205" s="2" t="s">
-        <v>67</v>
+        <v>1951</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>892</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.2">
@@ -7919,10 +8087,10 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" s="3" t="s">
-        <v>440</v>
+        <v>1953</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>908</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
@@ -9407,10 +9575,10 @@
     </row>
     <row r="404" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A404" s="3" t="s">
-        <v>456</v>
+        <v>1955</v>
       </c>
       <c r="B404" s="3" t="s">
-        <v>1137</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.2">
@@ -10058,7 +10226,7 @@
         <v>671</v>
       </c>
       <c r="B485" s="3" t="s">
-        <v>1238</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="486" spans="1:2" x14ac:dyDescent="0.2">
@@ -10583,10 +10751,10 @@
     </row>
     <row r="551" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A551" s="3" t="s">
-        <v>671</v>
+        <v>1957</v>
       </c>
       <c r="B551" s="3" t="s">
-        <v>1321</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="552" spans="1:2" x14ac:dyDescent="0.2">
@@ -10719,10 +10887,10 @@
     </row>
     <row r="568" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A568" s="2" t="s">
-        <v>1343</v>
+        <v>1959</v>
       </c>
       <c r="B568" s="2" t="s">
-        <v>1344</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="569" spans="1:2" x14ac:dyDescent="0.2">
@@ -10930,7 +11098,7 @@
         <v>1343</v>
       </c>
       <c r="B594" s="3" t="s">
-        <v>1380</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="595" spans="1:2" x14ac:dyDescent="0.2">
@@ -11119,10 +11287,10 @@
     </row>
     <row r="618" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A618" s="2" t="s">
-        <v>1302</v>
+        <v>1961</v>
       </c>
       <c r="B618" s="2" t="s">
-        <v>1407</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="619" spans="1:2" x14ac:dyDescent="0.2">
@@ -11938,7 +12106,7 @@
         <v>244</v>
       </c>
       <c r="B720" s="2" t="s">
-        <v>1545</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="721" spans="1:2" x14ac:dyDescent="0.2">
@@ -13146,7 +13314,7 @@
         <v>1763</v>
       </c>
       <c r="B871" s="3" t="s">
-        <v>1764</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="872" spans="1:2" x14ac:dyDescent="0.2">
@@ -13410,7 +13578,7 @@
         <v>1814</v>
       </c>
       <c r="B904" s="2" t="s">
-        <v>1815</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="905" spans="1:2" x14ac:dyDescent="0.2">
@@ -13490,7 +13658,7 @@
         <v>1829</v>
       </c>
       <c r="B914" s="2" t="s">
-        <v>1830</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="915" spans="1:2" x14ac:dyDescent="0.2">
@@ -14067,6 +14235,126 @@
       </c>
       <c r="B986" s="3" t="s">
         <v>1936</v>
+      </c>
+    </row>
+    <row r="987" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A987" s="2" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B987" s="2" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="988" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A988" s="3" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B988" s="3" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="989" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A989" s="2" t="s">
+        <v>1967</v>
+      </c>
+      <c r="B989" s="2" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="990" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A990" s="3" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B990" s="3" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="991" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A991" s="2" t="s">
+        <v>1971</v>
+      </c>
+      <c r="B991" s="2" t="s">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="992" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A992" s="3" t="s">
+        <v>1973</v>
+      </c>
+      <c r="B992" s="3" t="s">
+        <v>1974</v>
+      </c>
+    </row>
+    <row r="993" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A993" s="2" t="s">
+        <v>1975</v>
+      </c>
+      <c r="B993" s="2" t="s">
+        <v>1976</v>
+      </c>
+    </row>
+    <row r="994" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A994" s="3" t="s">
+        <v>1977</v>
+      </c>
+      <c r="B994" s="3" t="s">
+        <v>1978</v>
+      </c>
+    </row>
+    <row r="995" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A995" s="2" t="s">
+        <v>1979</v>
+      </c>
+      <c r="B995" s="2" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="996" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A996" s="3" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B996" s="3" t="s">
+        <v>1982</v>
+      </c>
+    </row>
+    <row r="997" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A997" s="2" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B997" s="2" t="s">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="998" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A998" s="3" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B998" s="3" t="s">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="999" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A999" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B999" s="2" t="s">
+        <v>1988</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1000" s="3" t="s">
+        <v>1989</v>
+      </c>
+      <c r="B1000" s="3" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1001" s="2" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B1001" s="2" t="s">
+        <v>1992</v>
       </c>
     </row>
   </sheetData>

</xml_diff>